<commit_message>
feat: add browser ai workspace UI and gateway transport handlers
</commit_message>
<xml_diff>
--- a/target_websites_sample.xlsx
+++ b/target_websites_sample.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="30.83203125" customWidth="1"/>
     <col min="2" max="2" width="24.83203125" customWidth="1"/>
@@ -425,10 +425,10 @@
     </row>
     <row r="2">
       <c r="A2" t="str">
-        <v>chatgpt.com</v>
+        <v>chat.example.com</v>
       </c>
       <c r="B2" t="str">
-        <v>ChatGPT</v>
+        <v>Example AI</v>
       </c>
       <c r="C2" t="str">
         <v>ui</v>
@@ -442,10 +442,10 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>ab.chatgpt.com</v>
+        <v>api.chat.example.com</v>
       </c>
       <c r="B3" t="str">
-        <v>ChatGPT</v>
+        <v>Example AI</v>
       </c>
       <c r="C3" t="str">
         <v>chat</v>
@@ -459,364 +459,24 @@
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>chat.openai.com</v>
+        <v>files.chat.example.com</v>
       </c>
       <c r="B4" t="str">
-        <v>ChatGPT</v>
+        <v>Example AI</v>
       </c>
       <c r="C4" t="str">
-        <v>chat</v>
+        <v>file</v>
       </c>
       <c r="D4" t="str">
         <v>TRUE</v>
       </c>
       <c r="E4" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="str">
-        <v>api.openai.com</v>
-      </c>
-      <c r="B5" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C5" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D5" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E5" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="str">
-        <v>files.oaiusercontent.com</v>
-      </c>
-      <c r="B6" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C6" t="str">
-        <v>file</v>
-      </c>
-      <c r="D6" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E6" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>oaiusercontent.com</v>
-      </c>
-      <c r="B7" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C7" t="str">
-        <v>file</v>
-      </c>
-      <c r="D7" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E7" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" t="str">
-        <v>oaistatic.com</v>
-      </c>
-      <c r="B8" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C8" t="str">
-        <v>file</v>
-      </c>
-      <c r="D8" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E8" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="str">
-        <v>cdn.oaistatic.com</v>
-      </c>
-      <c r="B9" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C9" t="str">
-        <v>file</v>
-      </c>
-      <c r="D9" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E9" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="str">
-        <v>ws.chatgpt.com</v>
-      </c>
-      <c r="B10" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C10" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D10" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E10" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="str">
-        <v>ws-api.chatgpt.com</v>
-      </c>
-      <c r="B11" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C11" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D11" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E11" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>realtime.chatgpt.com</v>
-      </c>
-      <c r="B12" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C12" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D12" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E12" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="str">
-        <v>openai.com</v>
-      </c>
-      <c r="B13" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C13" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D13" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E13" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="str">
-        <v>browser-gateway-openai.livekit.cloud</v>
-      </c>
-      <c r="B14" t="str">
-        <v>ChatGPT</v>
-      </c>
-      <c r="C14" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D14" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E14" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="str">
-        <v>claude.ai</v>
-      </c>
-      <c r="B15" t="str">
-        <v>Claude</v>
-      </c>
-      <c r="C15" t="str">
-        <v>ui</v>
-      </c>
-      <c r="D15" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E15" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="str">
-        <v>api.anthropic.com</v>
-      </c>
-      <c r="B16" t="str">
-        <v>Claude</v>
-      </c>
-      <c r="C16" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D16" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E16" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="str">
-        <v>files.claudeusercontent.com</v>
-      </c>
-      <c r="B17" t="str">
-        <v>Claude</v>
-      </c>
-      <c r="C17" t="str">
-        <v>file</v>
-      </c>
-      <c r="D17" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E17" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="str">
-        <v>cdn.claude.ai</v>
-      </c>
-      <c r="B18" t="str">
-        <v>Claude</v>
-      </c>
-      <c r="C18" t="str">
-        <v>file</v>
-      </c>
-      <c r="D18" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E18" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="str">
-        <v>anthropic.com</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Claude</v>
-      </c>
-      <c r="C19" t="str">
-        <v>ui</v>
-      </c>
-      <c r="D19" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E19" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="str">
-        <v>gemini.google.com</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Gemini</v>
-      </c>
-      <c r="C20" t="str">
-        <v>ui</v>
-      </c>
-      <c r="D20" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E20" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="str">
-        <v>clients6.google.com</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Gemini</v>
-      </c>
-      <c r="C21" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D21" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E21" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="str">
-        <v>generativelanguage.googleapis.com</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Gemini</v>
-      </c>
-      <c r="C22" t="str">
-        <v>chat</v>
-      </c>
-      <c r="D22" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E22" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="str">
-        <v>aistudio.google.com</v>
-      </c>
-      <c r="B23" t="str">
-        <v>Gemini</v>
-      </c>
-      <c r="C23" t="str">
-        <v>ui</v>
-      </c>
-      <c r="D23" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E23" t="str">
-        <v>FALSE</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="str">
-        <v>bard.google.com</v>
-      </c>
-      <c r="B24" t="str">
-        <v>Gemini</v>
-      </c>
-      <c r="C24" t="str">
-        <v>ui</v>
-      </c>
-      <c r="D24" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="E24" t="str">
         <v>FALSE</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>